<commit_message>
Reimport all page content with complete bullet lists and text
Reimport all 17 pages from nextrow.com to capture full content
including bullet lists, descriptions, and all text that was
previously missing from cards and service sections.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="108">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,6 +37,138 @@
     <t>url</t>
   </si>
   <si>
+    <t>ai-services.report.json</t>
+  </si>
+  <si>
+    <t>["hero-service","cards-accelerator","columns-casestudy","embed-calendar"]</t>
+  </si>
+  <si>
+    <t>ai-services</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>service-page</t>
+  </si>
+  <si>
+    <t>2026-05-11T17:55:01.980Z</t>
+  </si>
+  <si>
+    <t>AI Services - NextRow</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/ai-services</t>
+  </si>
+  <si>
+    <t>b2b-marketing.report.json</t>
+  </si>
+  <si>
+    <t>["hero-service","columns-valueprop","cards-accelerator","columns-casestudy","embed-calendar"]</t>
+  </si>
+  <si>
+    <t>b2b-marketing</t>
+  </si>
+  <si>
+    <t>2026-05-11T17:54:34.921Z</t>
+  </si>
+  <si>
+    <t>B2B Marketing - NextRow</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/b2b-marketing</t>
+  </si>
+  <si>
+    <t>blog.report.json</t>
+  </si>
+  <si>
+    <t>["cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","form","form"]</t>
+  </si>
+  <si>
+    <t>blog</t>
+  </si>
+  <si>
+    <t>standard-page</t>
+  </si>
+  <si>
+    <t>2026-05-11T09:07:45.275Z</t>
+  </si>
+  <si>
+    <t>Insights - NextRow</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/blog</t>
+  </si>
+  <si>
+    <t>cloud-services.report.json</t>
+  </si>
+  <si>
+    <t>["cards-accelerator","cards-accelerator"]</t>
+  </si>
+  <si>
+    <t>cloud-services</t>
+  </si>
+  <si>
+    <t>2026-05-11T17:55:08.599Z</t>
+  </si>
+  <si>
+    <t>Cloud Services - NextRow</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/cloud-services</t>
+  </si>
+  <si>
+    <t>contact-us.report.json</t>
+  </si>
+  <si>
+    <t>["cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","form"]</t>
+  </si>
+  <si>
+    <t>contact-us</t>
+  </si>
+  <si>
+    <t>2026-05-11T09:07:38.424Z</t>
+  </si>
+  <si>
+    <t>Contact Us - NextRow</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/contact-us</t>
+  </si>
+  <si>
+    <t>content-supply-chain.report.json</t>
+  </si>
+  <si>
+    <t>content-supply-chain</t>
+  </si>
+  <si>
+    <t>2026-05-11T17:54:49.872Z</t>
+  </si>
+  <si>
+    <t>Content Supply Chain - NextRow</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/content-supply-chain</t>
+  </si>
+  <si>
+    <t>cyber-security.report.json</t>
+  </si>
+  <si>
+    <t>["cards-accelerator"]</t>
+  </si>
+  <si>
+    <t>cyber-security</t>
+  </si>
+  <si>
+    <t>2026-05-11T17:55:22.890Z</t>
+  </si>
+  <si>
+    <t>Cyber Security - NextRow</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/cyber-security</t>
+  </si>
+  <si>
     <t>index.report.json</t>
   </si>
   <si>
@@ -46,19 +178,163 @@
     <t>index</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-05-11T08:31:19.694Z</t>
+    <t>2026-05-11T17:55:48.281Z</t>
   </si>
   <si>
     <t>NextRow Digital: Driving Business Growth Effectively - NextRow</t>
   </si>
   <si>
     <t>https://www.nextrow.com/</t>
+  </si>
+  <si>
+    <t>koru.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>koru</t>
+  </si>
+  <si>
+    <t>product-page</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:57:38.728Z</t>
+  </si>
+  <si>
+    <t>Koru - NextRow</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/koru</t>
+  </si>
+  <si>
+    <t>martech-services.report.json</t>
+  </si>
+  <si>
+    <t>martech-services</t>
+  </si>
+  <si>
+    <t>2026-05-11T17:54:55.575Z</t>
+  </si>
+  <si>
+    <t>MarTech Services | MarTech Business Solutions | NextRow Digital</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/martech-services</t>
+  </si>
+  <si>
+    <t>partners.report.json</t>
+  </si>
+  <si>
+    <t>["cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner","cards-partner"]</t>
+  </si>
+  <si>
+    <t>partners</t>
+  </si>
+  <si>
+    <t>2026-05-11T09:07:31.026Z</t>
+  </si>
+  <si>
+    <t>Partners - NextRow</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/partners</t>
+  </si>
+  <si>
+    <t>privacy-policy.report.json</t>
+  </si>
+  <si>
+    <t>privacy-policy</t>
+  </si>
+  <si>
+    <t>2026-05-11T09:07:57.659Z</t>
+  </si>
+  <si>
+    <t>Privacy Policy - NextRow</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/privacy-policy</t>
+  </si>
+  <si>
+    <t>quiptag.report.json</t>
+  </si>
+  <si>
+    <t>["hero-product","columns-casestudy","embed-video","columns-stats","embed-calendar"]</t>
+  </si>
+  <si>
+    <t>quiptag</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:57:32.564Z</t>
+  </si>
+  <si>
+    <t>QuipTag: Accelerate Your Content Velocity - NextRow</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/quiptag</t>
+  </si>
+  <si>
+    <t>training.report.json</t>
+  </si>
+  <si>
+    <t>training</t>
+  </si>
+  <si>
+    <t>2026-05-11T09:07:51.660Z</t>
+  </si>
+  <si>
+    <t>AEM Training | Adobe Analytics Training | NextRow Digital</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/training</t>
+  </si>
+  <si>
+    <t>unified-customer-experience.report.json</t>
+  </si>
+  <si>
+    <t>unified-customer-experience</t>
+  </si>
+  <si>
+    <t>2026-05-11T17:54:43.006Z</t>
+  </si>
+  <si>
+    <t>Unified Customer Experience - NextRow</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/unified-customer-experience</t>
+  </si>
+  <si>
+    <t>workday-services.report.json</t>
+  </si>
+  <si>
+    <t>workday-services</t>
+  </si>
+  <si>
+    <t>2026-05-11T17:55:15.930Z</t>
+  </si>
+  <si>
+    <t>Workday Services - NextRow</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/workday-services</t>
+  </si>
+  <si>
+    <t>snowflake-services/cloud-data-analytics.report.json</t>
+  </si>
+  <si>
+    <t>snowflake-services/cloud-data-analytics</t>
+  </si>
+  <si>
+    <t>2026-05-11T17:55:29.826Z</t>
+  </si>
+  <si>
+    <t>Cloud Data Analytics - NextRow</t>
+  </si>
+  <si>
+    <t>https://www.nextrow.com/snowflake-services/cloud-data-analytics</t>
   </si>
 </sst>
 </file>
@@ -447,16 +723,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="7" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="41" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -509,6 +783,422 @@
       </c>
       <c r="H2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" t="s">
+        <v>50</v>
+      </c>
+      <c r="H8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>55</v>
+      </c>
+      <c r="F9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" t="s">
+        <v>57</v>
+      </c>
+      <c r="H9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F10" t="s">
+        <v>63</v>
+      </c>
+      <c r="G10" t="s">
+        <v>64</v>
+      </c>
+      <c r="H10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" t="s">
+        <v>68</v>
+      </c>
+      <c r="G11" t="s">
+        <v>69</v>
+      </c>
+      <c r="H11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" t="s">
+        <v>75</v>
+      </c>
+      <c r="H12" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
+        <v>78</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" t="s">
+        <v>80</v>
+      </c>
+      <c r="H13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" t="s">
+        <v>84</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>62</v>
+      </c>
+      <c r="F14" t="s">
+        <v>85</v>
+      </c>
+      <c r="G14" t="s">
+        <v>86</v>
+      </c>
+      <c r="H14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" t="s">
+        <v>89</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F15" t="s">
+        <v>90</v>
+      </c>
+      <c r="G15" t="s">
+        <v>91</v>
+      </c>
+      <c r="H15" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>93</v>
+      </c>
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" t="s">
+        <v>95</v>
+      </c>
+      <c r="G16" t="s">
+        <v>96</v>
+      </c>
+      <c r="H16" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>98</v>
+      </c>
+      <c r="B17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" t="s">
+        <v>99</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" t="s">
+        <v>100</v>
+      </c>
+      <c r="G17" t="s">
+        <v>101</v>
+      </c>
+      <c r="H17" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" t="s">
+        <v>104</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" t="s">
+        <v>105</v>
+      </c>
+      <c r="G18" t="s">
+        <v>106</v>
+      </c>
+      <c r="H18" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>